<commit_message>
Buen progreso, documento bastante avanzado
</commit_message>
<xml_diff>
--- a/Serrano-Jorge/source/Results/brassica.xlsx
+++ b/Serrano-Jorge/source/Results/brassica.xlsx
@@ -13,7 +13,73 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+  <si>
+    <t>CaliQ</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CUSTOM</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CaliQ</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CUSTOM</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
   <si>
     <t>CaliQ</t>
   </si>
@@ -66,7 +132,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -76,14 +142,22 @@
     </border>
     <border/>
     <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -111,14 +185,14 @@
     <row r="1">
       <c r="A1" s="0"/>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C1" s="0"/>
       <c r="D1" s="0"/>
       <c r="E1" s="0"/>
       <c r="F1" s="0"/>
       <c r="G1" s="0" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="H1" s="0"/>
       <c r="I1" s="0"/>
@@ -126,32 +200,32 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="F2" s="0"/>
       <c r="G2" s="0" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Commit porque me da miedo perder los cambios
</commit_message>
<xml_diff>
--- a/Serrano-Jorge/source/Results/brassica.xlsx
+++ b/Serrano-Jorge/source/Results/brassica.xlsx
@@ -13,7 +13,205 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
+  <si>
+    <t>CaliQ</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CUSTOM</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CaliQ</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CUSTOM</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CaliQ</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CUSTOM</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CaliQ</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CUSTOM</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CaliQ</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CUSTOM</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CaliQ</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
+  <si>
+    <t>CUSTOM</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>PSNR</t>
+  </si>
+  <si>
+    <t>SSIM</t>
+  </si>
   <si>
     <t>CaliQ</t>
   </si>
@@ -132,7 +330,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -146,11 +344,23 @@
     <border/>
     <border/>
     <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true"/>
@@ -158,6 +368,18 @@
     <xf numFmtId="22" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -185,14 +407,14 @@
     <row r="1">
       <c r="A1" s="0"/>
       <c r="B1" s="0" t="s">
-        <v>23</v>
+        <v>89</v>
       </c>
       <c r="C1" s="0"/>
       <c r="D1" s="0"/>
       <c r="E1" s="0"/>
       <c r="F1" s="0"/>
       <c r="G1" s="0" t="s">
-        <v>28</v>
+        <v>94</v>
       </c>
       <c r="H1" s="0"/>
       <c r="I1" s="0"/>
@@ -200,32 +422,32 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>24</v>
+        <v>90</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>27</v>
+        <v>93</v>
       </c>
       <c r="F2" s="0"/>
       <c r="G2" s="0" t="s">
-        <v>29</v>
+        <v>95</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>30</v>
+        <v>96</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>31</v>
+        <v>97</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>32</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3">

</xml_diff>